<commit_message>
Fix static charts and Excel negatives
- Horizontal bars now label the category axis instead of numbers
- Series on a right-hand axis get their own scale in PNG charts
- Excel bar series set invertIfNegative=false so negative values plot below zero
- Hex colours and stacked bars render as configured
</commit_message>
<xml_diff>
--- a/excel/appeals-friction-radar_dashboard.xlsx
+++ b/excel/appeals-friction-radar_dashboard.xlsx
@@ -288,6 +288,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_stages'!$A$2:$A$6</f>
@@ -312,6 +313,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -340,6 +342,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -448,6 +451,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_by_type'!$A$2:$A$6</f>
@@ -476,6 +480,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_by_type'!$A$2:$A$6</f>
@@ -500,6 +505,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -513,6 +519,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -565,6 +572,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_by_type_2'!$A$2:$A$6</f>
@@ -589,6 +597,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -617,6 +626,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -742,6 +752,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_friction'!$A$2:$A$5</f>
@@ -766,6 +777,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -793,6 +805,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <valAx>
         <axId val="200"/>
@@ -872,6 +885,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_doc_gap'!$A$2:$A$3</f>
@@ -900,6 +914,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_doc_gap'!$A$2:$A$3</f>
@@ -928,6 +943,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_doc_gap'!$A$2:$A$3</f>
@@ -952,6 +968,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -965,6 +982,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1017,6 +1035,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_rework'!$A$2:$A$3</f>
@@ -1045,6 +1064,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_rework'!$A$2:$A$3</f>
@@ -1069,6 +1089,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -1082,6 +1103,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1211,6 +1233,7 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
             <numRef>
               <f>'q_monthly'!$A$2:$A$10</f>
@@ -1235,6 +1258,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -1262,6 +1286,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <valAx>
         <axId val="200"/>

</xml_diff>